<commit_message>
feat: enhance hybrid recommendation engine with realistic data patterns and improved CF scaling
</commit_message>
<xml_diff>
--- a/data rating.xlsx
+++ b/data rating.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5260,6 +5260,1972 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr"/>
+      <c r="C235" t="n">
+        <v>4</v>
+      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr"/>
+      <c r="C236" t="n">
+        <v>4</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1</v>
+      </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr"/>
+      <c r="C237" t="n">
+        <v>5</v>
+      </c>
+      <c r="D237" t="n">
+        <v>34</v>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr"/>
+      <c r="C238" t="n">
+        <v>5</v>
+      </c>
+      <c r="D238" t="n">
+        <v>4</v>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr"/>
+      <c r="C239" t="n">
+        <v>5</v>
+      </c>
+      <c r="D239" t="n">
+        <v>36</v>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr"/>
+      <c r="C240" t="n">
+        <v>4</v>
+      </c>
+      <c r="D240" t="n">
+        <v>14</v>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr"/>
+      <c r="C241" t="n">
+        <v>4</v>
+      </c>
+      <c r="D241" t="n">
+        <v>17</v>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr"/>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr"/>
+      <c r="C242" t="n">
+        <v>4</v>
+      </c>
+      <c r="D242" t="n">
+        <v>20</v>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr"/>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr"/>
+      <c r="C243" t="n">
+        <v>5</v>
+      </c>
+      <c r="D243" t="n">
+        <v>24</v>
+      </c>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Traveler_Active_1</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr"/>
+      <c r="C244" t="n">
+        <v>5</v>
+      </c>
+      <c r="D244" t="n">
+        <v>27</v>
+      </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr"/>
+      <c r="C245" t="n">
+        <v>5</v>
+      </c>
+      <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr"/>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr"/>
+      <c r="C246" t="n">
+        <v>4</v>
+      </c>
+      <c r="D246" t="n">
+        <v>35</v>
+      </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr"/>
+      <c r="C247" t="n">
+        <v>5</v>
+      </c>
+      <c r="D247" t="n">
+        <v>8</v>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr"/>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr"/>
+      <c r="C248" t="n">
+        <v>4</v>
+      </c>
+      <c r="D248" t="n">
+        <v>13</v>
+      </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr"/>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr"/>
+      <c r="C249" t="n">
+        <v>5</v>
+      </c>
+      <c r="D249" t="n">
+        <v>21</v>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr"/>
+      <c r="C250" t="n">
+        <v>4</v>
+      </c>
+      <c r="D250" t="n">
+        <v>23</v>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr"/>
+      <c r="C251" t="n">
+        <v>4</v>
+      </c>
+      <c r="D251" t="n">
+        <v>25</v>
+      </c>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr"/>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr"/>
+      <c r="C252" t="n">
+        <v>4</v>
+      </c>
+      <c r="D252" t="n">
+        <v>27</v>
+      </c>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr"/>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr"/>
+      <c r="C253" t="n">
+        <v>5</v>
+      </c>
+      <c r="D253" t="n">
+        <v>28</v>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr"/>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Traveler_Active_2</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr"/>
+      <c r="C254" t="n">
+        <v>4</v>
+      </c>
+      <c r="D254" t="n">
+        <v>30</v>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr"/>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr"/>
+      <c r="C255" t="n">
+        <v>5</v>
+      </c>
+      <c r="D255" t="n">
+        <v>1</v>
+      </c>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr"/>
+      <c r="C256" t="n">
+        <v>4</v>
+      </c>
+      <c r="D256" t="n">
+        <v>34</v>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr"/>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr"/>
+      <c r="C257" t="n">
+        <v>5</v>
+      </c>
+      <c r="D257" t="n">
+        <v>35</v>
+      </c>
+      <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr"/>
+      <c r="C258" t="n">
+        <v>5</v>
+      </c>
+      <c r="D258" t="n">
+        <v>4</v>
+      </c>
+      <c r="E258" t="inlineStr"/>
+      <c r="F258" t="inlineStr"/>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr"/>
+      <c r="C259" t="n">
+        <v>5</v>
+      </c>
+      <c r="D259" t="n">
+        <v>10</v>
+      </c>
+      <c r="E259" t="inlineStr"/>
+      <c r="F259" t="inlineStr"/>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr"/>
+      <c r="C260" t="n">
+        <v>5</v>
+      </c>
+      <c r="D260" t="n">
+        <v>14</v>
+      </c>
+      <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr"/>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr"/>
+      <c r="C261" t="n">
+        <v>5</v>
+      </c>
+      <c r="D261" t="n">
+        <v>25</v>
+      </c>
+      <c r="E261" t="inlineStr"/>
+      <c r="F261" t="inlineStr"/>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr"/>
+      <c r="C262" t="n">
+        <v>5</v>
+      </c>
+      <c r="D262" t="n">
+        <v>27</v>
+      </c>
+      <c r="E262" t="inlineStr"/>
+      <c r="F262" t="inlineStr"/>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Traveler_Active_3</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr"/>
+      <c r="C263" t="n">
+        <v>4</v>
+      </c>
+      <c r="D263" t="n">
+        <v>31</v>
+      </c>
+      <c r="E263" t="inlineStr"/>
+      <c r="F263" t="inlineStr"/>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr"/>
+      <c r="C264" t="n">
+        <v>4</v>
+      </c>
+      <c r="D264" t="inlineStr"/>
+      <c r="E264" t="inlineStr"/>
+      <c r="F264" t="inlineStr"/>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr"/>
+      <c r="C265" t="n">
+        <v>4</v>
+      </c>
+      <c r="D265" t="n">
+        <v>38</v>
+      </c>
+      <c r="E265" t="inlineStr"/>
+      <c r="F265" t="inlineStr"/>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr"/>
+      <c r="C266" t="n">
+        <v>4</v>
+      </c>
+      <c r="D266" t="n">
+        <v>9</v>
+      </c>
+      <c r="E266" t="inlineStr"/>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr"/>
+      <c r="C267" t="n">
+        <v>5</v>
+      </c>
+      <c r="D267" t="n">
+        <v>11</v>
+      </c>
+      <c r="E267" t="inlineStr"/>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr"/>
+      <c r="C268" t="n">
+        <v>4</v>
+      </c>
+      <c r="D268" t="n">
+        <v>13</v>
+      </c>
+      <c r="E268" t="inlineStr"/>
+      <c r="F268" t="inlineStr"/>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr"/>
+      <c r="C269" t="n">
+        <v>4</v>
+      </c>
+      <c r="D269" t="n">
+        <v>24</v>
+      </c>
+      <c r="E269" t="inlineStr"/>
+      <c r="F269" t="inlineStr"/>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr"/>
+      <c r="C270" t="n">
+        <v>4</v>
+      </c>
+      <c r="D270" t="n">
+        <v>25</v>
+      </c>
+      <c r="E270" t="inlineStr"/>
+      <c r="F270" t="inlineStr"/>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr"/>
+      <c r="C271" t="n">
+        <v>5</v>
+      </c>
+      <c r="D271" t="n">
+        <v>28</v>
+      </c>
+      <c r="E271" t="inlineStr"/>
+      <c r="F271" t="inlineStr"/>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Traveler_Active_4</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr"/>
+      <c r="C272" t="n">
+        <v>4</v>
+      </c>
+      <c r="D272" t="n">
+        <v>30</v>
+      </c>
+      <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr"/>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr"/>
+      <c r="C273" t="n">
+        <v>4</v>
+      </c>
+      <c r="D273" t="inlineStr"/>
+      <c r="E273" t="inlineStr"/>
+      <c r="F273" t="inlineStr"/>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr"/>
+      <c r="C274" t="n">
+        <v>5</v>
+      </c>
+      <c r="D274" t="n">
+        <v>1</v>
+      </c>
+      <c r="E274" t="inlineStr"/>
+      <c r="F274" t="inlineStr"/>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr"/>
+      <c r="C275" t="n">
+        <v>5</v>
+      </c>
+      <c r="D275" t="n">
+        <v>7</v>
+      </c>
+      <c r="E275" t="inlineStr"/>
+      <c r="F275" t="inlineStr"/>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr"/>
+      <c r="C276" t="n">
+        <v>5</v>
+      </c>
+      <c r="D276" t="n">
+        <v>10</v>
+      </c>
+      <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr"/>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr"/>
+      <c r="C277" t="n">
+        <v>5</v>
+      </c>
+      <c r="D277" t="n">
+        <v>12</v>
+      </c>
+      <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr"/>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr"/>
+      <c r="C278" t="n">
+        <v>5</v>
+      </c>
+      <c r="D278" t="n">
+        <v>22</v>
+      </c>
+      <c r="E278" t="inlineStr"/>
+      <c r="F278" t="inlineStr"/>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr"/>
+      <c r="C279" t="n">
+        <v>4</v>
+      </c>
+      <c r="D279" t="n">
+        <v>23</v>
+      </c>
+      <c r="E279" t="inlineStr"/>
+      <c r="F279" t="inlineStr"/>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr"/>
+      <c r="C280" t="n">
+        <v>4</v>
+      </c>
+      <c r="D280" t="n">
+        <v>24</v>
+      </c>
+      <c r="E280" t="inlineStr"/>
+      <c r="F280" t="inlineStr"/>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Traveler_Active_5</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr"/>
+      <c r="C281" t="n">
+        <v>4</v>
+      </c>
+      <c r="D281" t="n">
+        <v>29</v>
+      </c>
+      <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr"/>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr"/>
+      <c r="C282" t="n">
+        <v>5</v>
+      </c>
+      <c r="D282" t="n">
+        <v>37</v>
+      </c>
+      <c r="E282" t="inlineStr"/>
+      <c r="F282" t="inlineStr"/>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr"/>
+      <c r="C283" t="n">
+        <v>4</v>
+      </c>
+      <c r="D283" t="n">
+        <v>7</v>
+      </c>
+      <c r="E283" t="inlineStr"/>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr"/>
+      <c r="C284" t="n">
+        <v>4</v>
+      </c>
+      <c r="D284" t="n">
+        <v>14</v>
+      </c>
+      <c r="E284" t="inlineStr"/>
+      <c r="F284" t="inlineStr"/>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr"/>
+      <c r="C285" t="n">
+        <v>4</v>
+      </c>
+      <c r="D285" t="n">
+        <v>17</v>
+      </c>
+      <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr"/>
+      <c r="C286" t="n">
+        <v>5</v>
+      </c>
+      <c r="D286" t="n">
+        <v>19</v>
+      </c>
+      <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr"/>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr"/>
+      <c r="C287" t="n">
+        <v>4</v>
+      </c>
+      <c r="D287" t="n">
+        <v>20</v>
+      </c>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr"/>
+      <c r="C288" t="n">
+        <v>4</v>
+      </c>
+      <c r="D288" t="n">
+        <v>21</v>
+      </c>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Traveler_Active_6</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr"/>
+      <c r="C289" t="n">
+        <v>4</v>
+      </c>
+      <c r="D289" t="n">
+        <v>23</v>
+      </c>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr"/>
+      <c r="C290" t="n">
+        <v>4</v>
+      </c>
+      <c r="D290" t="n">
+        <v>4</v>
+      </c>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr"/>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr"/>
+      <c r="C291" t="n">
+        <v>4</v>
+      </c>
+      <c r="D291" t="n">
+        <v>39</v>
+      </c>
+      <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr"/>
+      <c r="C292" t="n">
+        <v>4</v>
+      </c>
+      <c r="D292" t="n">
+        <v>7</v>
+      </c>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr"/>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr"/>
+      <c r="C293" t="n">
+        <v>4</v>
+      </c>
+      <c r="D293" t="n">
+        <v>10</v>
+      </c>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr"/>
+      <c r="C294" t="n">
+        <v>4</v>
+      </c>
+      <c r="D294" t="n">
+        <v>16</v>
+      </c>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr"/>
+      <c r="C295" t="n">
+        <v>4</v>
+      </c>
+      <c r="D295" t="n">
+        <v>17</v>
+      </c>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr"/>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr"/>
+      <c r="C296" t="n">
+        <v>5</v>
+      </c>
+      <c r="D296" t="n">
+        <v>20</v>
+      </c>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr"/>
+      <c r="C297" t="n">
+        <v>5</v>
+      </c>
+      <c r="D297" t="n">
+        <v>21</v>
+      </c>
+      <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Traveler_Active_7</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr"/>
+      <c r="C298" t="n">
+        <v>5</v>
+      </c>
+      <c r="D298" t="n">
+        <v>29</v>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr"/>
+      <c r="C299" t="n">
+        <v>4</v>
+      </c>
+      <c r="D299" t="n">
+        <v>1</v>
+      </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr"/>
+      <c r="C300" t="n">
+        <v>5</v>
+      </c>
+      <c r="D300" t="n">
+        <v>34</v>
+      </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr"/>
+      <c r="C301" t="n">
+        <v>5</v>
+      </c>
+      <c r="D301" t="n">
+        <v>39</v>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr"/>
+      <c r="C302" t="n">
+        <v>4</v>
+      </c>
+      <c r="D302" t="n">
+        <v>7</v>
+      </c>
+      <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr"/>
+      <c r="C303" t="n">
+        <v>4</v>
+      </c>
+      <c r="D303" t="n">
+        <v>14</v>
+      </c>
+      <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr"/>
+      <c r="C304" t="n">
+        <v>5</v>
+      </c>
+      <c r="D304" t="n">
+        <v>16</v>
+      </c>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr"/>
+      <c r="C305" t="n">
+        <v>4</v>
+      </c>
+      <c r="D305" t="n">
+        <v>17</v>
+      </c>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr"/>
+      <c r="C306" t="n">
+        <v>5</v>
+      </c>
+      <c r="D306" t="n">
+        <v>19</v>
+      </c>
+      <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr"/>
+      <c r="C307" t="n">
+        <v>5</v>
+      </c>
+      <c r="D307" t="n">
+        <v>20</v>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Traveler_Active_8</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr"/>
+      <c r="C308" t="n">
+        <v>4</v>
+      </c>
+      <c r="D308" t="n">
+        <v>21</v>
+      </c>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr"/>
+      <c r="C309" t="n">
+        <v>4</v>
+      </c>
+      <c r="D309" t="n">
+        <v>35</v>
+      </c>
+      <c r="E309" t="inlineStr"/>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr"/>
+      <c r="C310" t="n">
+        <v>5</v>
+      </c>
+      <c r="D310" t="n">
+        <v>36</v>
+      </c>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr"/>
+      <c r="C311" t="n">
+        <v>4</v>
+      </c>
+      <c r="D311" t="n">
+        <v>7</v>
+      </c>
+      <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr"/>
+      <c r="C312" t="n">
+        <v>4</v>
+      </c>
+      <c r="D312" t="n">
+        <v>39</v>
+      </c>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr"/>
+      <c r="C313" t="n">
+        <v>4</v>
+      </c>
+      <c r="D313" t="n">
+        <v>40</v>
+      </c>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr"/>
+      <c r="C314" t="n">
+        <v>4</v>
+      </c>
+      <c r="D314" t="n">
+        <v>9</v>
+      </c>
+      <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr"/>
+      <c r="C315" t="n">
+        <v>4</v>
+      </c>
+      <c r="D315" t="n">
+        <v>14</v>
+      </c>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr"/>
+      <c r="C316" t="n">
+        <v>5</v>
+      </c>
+      <c r="D316" t="n">
+        <v>16</v>
+      </c>
+      <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr"/>
+      <c r="C317" t="n">
+        <v>5</v>
+      </c>
+      <c r="D317" t="n">
+        <v>17</v>
+      </c>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Traveler_Active_9</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr"/>
+      <c r="C318" t="n">
+        <v>5</v>
+      </c>
+      <c r="D318" t="n">
+        <v>21</v>
+      </c>
+      <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr"/>
+      <c r="C319" t="n">
+        <v>4</v>
+      </c>
+      <c r="D319" t="n">
+        <v>4</v>
+      </c>
+      <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr"/>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr"/>
+      <c r="C320" t="n">
+        <v>5</v>
+      </c>
+      <c r="D320" t="n">
+        <v>38</v>
+      </c>
+      <c r="E320" t="inlineStr"/>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr"/>
+      <c r="C321" t="n">
+        <v>4</v>
+      </c>
+      <c r="D321" t="n">
+        <v>7</v>
+      </c>
+      <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr"/>
+      <c r="C322" t="n">
+        <v>5</v>
+      </c>
+      <c r="D322" t="n">
+        <v>40</v>
+      </c>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr"/>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr"/>
+      <c r="C323" t="n">
+        <v>5</v>
+      </c>
+      <c r="D323" t="n">
+        <v>9</v>
+      </c>
+      <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr"/>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr"/>
+      <c r="C324" t="n">
+        <v>5</v>
+      </c>
+      <c r="D324" t="n">
+        <v>16</v>
+      </c>
+      <c r="E324" t="inlineStr"/>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr"/>
+      <c r="C325" t="n">
+        <v>4</v>
+      </c>
+      <c r="D325" t="n">
+        <v>17</v>
+      </c>
+      <c r="E325" t="inlineStr"/>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr"/>
+      <c r="C326" t="n">
+        <v>5</v>
+      </c>
+      <c r="D326" t="n">
+        <v>19</v>
+      </c>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr"/>
+      <c r="C327" t="n">
+        <v>5</v>
+      </c>
+      <c r="D327" t="n">
+        <v>20</v>
+      </c>
+      <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Traveler_Active_10</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr"/>
+      <c r="C328" t="n">
+        <v>5</v>
+      </c>
+      <c r="D328" t="n">
+        <v>21</v>
+      </c>
+      <c r="E328" t="inlineStr"/>
+      <c r="F328" t="inlineStr"/>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Pengalaman yang sangat menyenangkan, direkomendasikan!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>